<commit_message>
Updated the new activities
</commit_message>
<xml_diff>
--- a/1234567.xlsx
+++ b/1234567.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Chirag Bhalla\Documents\Minor-project cap-776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AAFDC21-FAB6-42E1-90D5-100BB843776E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3225ECE8-67D9-4352-A572-E49A41FAF7FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="73">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -235,6 +235,27 @@
   </si>
   <si>
     <t>went for running and gym, working on myself, prepared for coding test</t>
+  </si>
+  <si>
+    <t>Excellent</t>
+  </si>
+  <si>
+    <t>Very Satisfied</t>
+  </si>
+  <si>
+    <t>Unsatisfied</t>
+  </si>
+  <si>
+    <t>went for 5k run</t>
+  </si>
+  <si>
+    <t>gave body some rest and prepared for next week</t>
+  </si>
+  <si>
+    <t>worked and studied in library</t>
+  </si>
+  <si>
+    <t>prepared for ca and worked on coding</t>
   </si>
 </sst>
 </file>
@@ -1256,92 +1277,188 @@
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A11" s="13"/>
-      <c r="B11" s="14"/>
-      <c r="C11" s="14"/>
-      <c r="D11" s="14"/>
-      <c r="E11" s="14"/>
-      <c r="F11" s="14"/>
-      <c r="G11" s="14"/>
-      <c r="H11" s="14"/>
-      <c r="I11" s="15" t="str">
+      <c r="A11" s="13">
+        <v>46256</v>
+      </c>
+      <c r="B11" s="14">
+        <v>450</v>
+      </c>
+      <c r="C11" s="14">
+        <v>120</v>
+      </c>
+      <c r="D11" s="14">
+        <v>120</v>
+      </c>
+      <c r="E11" s="14">
+        <v>90</v>
+      </c>
+      <c r="F11" s="14">
+        <v>0</v>
+      </c>
+      <c r="G11" s="14">
+        <v>0</v>
+      </c>
+      <c r="H11" s="14">
+        <v>120</v>
+      </c>
+      <c r="I11" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J11" s="15" t="str">
+        <v>900</v>
+      </c>
+      <c r="J11" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K11" s="16"/>
-      <c r="L11" s="16"/>
-      <c r="M11" s="16"/>
-      <c r="N11" s="17"/>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A12" s="13"/>
-      <c r="B12" s="14"/>
-      <c r="C12" s="14"/>
-      <c r="D12" s="14"/>
-      <c r="E12" s="14"/>
-      <c r="F12" s="14"/>
-      <c r="G12" s="14"/>
-      <c r="H12" s="14"/>
-      <c r="I12" s="15" t="str">
+        <v>540</v>
+      </c>
+      <c r="K11" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="L11" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="M11" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N11" s="17" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A12" s="13">
+        <v>46257</v>
+      </c>
+      <c r="B12" s="14">
+        <v>420</v>
+      </c>
+      <c r="C12" s="14">
+        <v>120</v>
+      </c>
+      <c r="D12" s="14">
+        <v>180</v>
+      </c>
+      <c r="E12" s="14">
+        <v>60</v>
+      </c>
+      <c r="F12" s="14">
+        <v>0</v>
+      </c>
+      <c r="G12" s="14">
+        <v>0</v>
+      </c>
+      <c r="H12" s="14">
+        <v>120</v>
+      </c>
+      <c r="I12" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J12" s="15" t="str">
+        <v>900</v>
+      </c>
+      <c r="J12" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K12" s="16"/>
-      <c r="L12" s="16"/>
-      <c r="M12" s="16"/>
-      <c r="N12" s="17"/>
+        <v>540</v>
+      </c>
+      <c r="K12" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L12" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="M12" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N12" s="17" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A13" s="13"/>
-      <c r="B13" s="14"/>
-      <c r="C13" s="14"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="14"/>
-      <c r="F13" s="14"/>
-      <c r="G13" s="14"/>
-      <c r="H13" s="14"/>
-      <c r="I13" s="15" t="str">
+      <c r="A13" s="13">
+        <v>46258</v>
+      </c>
+      <c r="B13" s="14">
+        <v>400</v>
+      </c>
+      <c r="C13" s="14">
+        <v>90</v>
+      </c>
+      <c r="D13" s="14">
+        <v>80</v>
+      </c>
+      <c r="E13" s="14">
+        <v>90</v>
+      </c>
+      <c r="F13" s="14">
+        <v>250</v>
+      </c>
+      <c r="G13" s="14">
+        <v>5</v>
+      </c>
+      <c r="H13" s="14">
+        <v>180</v>
+      </c>
+      <c r="I13" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J13" s="15" t="str">
+        <v>1090</v>
+      </c>
+      <c r="J13" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K13" s="16"/>
-      <c r="L13" s="16"/>
-      <c r="M13" s="16"/>
-      <c r="N13" s="17"/>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A14" s="13"/>
-      <c r="B14" s="14"/>
-      <c r="C14" s="14"/>
-      <c r="D14" s="14"/>
-      <c r="E14" s="14"/>
-      <c r="F14" s="14"/>
-      <c r="G14" s="14"/>
-      <c r="H14" s="14"/>
-      <c r="I14" s="15" t="str">
+        <v>350</v>
+      </c>
+      <c r="K13" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="L13" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="M13" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N13" s="17" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A14" s="13">
+        <v>46259</v>
+      </c>
+      <c r="B14" s="14">
+        <v>380</v>
+      </c>
+      <c r="C14" s="14">
+        <v>90</v>
+      </c>
+      <c r="D14" s="14">
+        <v>60</v>
+      </c>
+      <c r="E14" s="14">
+        <v>120</v>
+      </c>
+      <c r="F14" s="14">
+        <v>250</v>
+      </c>
+      <c r="G14" s="14">
+        <v>5</v>
+      </c>
+      <c r="H14" s="14">
+        <v>180</v>
+      </c>
+      <c r="I14" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J14" s="15" t="str">
+        <v>1080</v>
+      </c>
+      <c r="J14" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K14" s="16"/>
-      <c r="L14" s="16"/>
-      <c r="M14" s="16"/>
-      <c r="N14" s="17"/>
+        <v>360</v>
+      </c>
+      <c r="K14" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="L14" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="M14" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N14" s="17" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" s="13"/>

</xml_diff>

<commit_message>
Updated the entrygit add 1234567.xlsx
</commit_message>
<xml_diff>
--- a/1234567.xlsx
+++ b/1234567.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Chirag Bhalla\Documents\Minor-project cap-776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3FF0159-42E8-4106-83B4-64C744320F75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{297D2A97-3983-4DBE-87FE-70130713BF3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="16305" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="89">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -271,6 +271,39 @@
   </si>
   <si>
     <t>started with python file management and worked on pandas</t>
+  </si>
+  <si>
+    <t>starting with analytical skills</t>
+  </si>
+  <si>
+    <t>did homework</t>
+  </si>
+  <si>
+    <t>registered for a hackathon</t>
+  </si>
+  <si>
+    <t>did homeworkl</t>
+  </si>
+  <si>
+    <t>went to meet friends felt refreshing</t>
+  </si>
+  <si>
+    <t>missed 2 classes due to waking up late</t>
+  </si>
+  <si>
+    <t xml:space="preserve">started with cpp file handling </t>
+  </si>
+  <si>
+    <t>not feeling well, probably viral</t>
+  </si>
+  <si>
+    <t>rested and worked on project</t>
+  </si>
+  <si>
+    <t xml:space="preserve">still not feeling well just did rest </t>
+  </si>
+  <si>
+    <t>didn’t do much work and rested a bit</t>
   </si>
 </sst>
 </file>
@@ -1709,267 +1742,553 @@
       <c r="A20" s="13">
         <v>46265</v>
       </c>
-      <c r="B20" s="14"/>
-      <c r="C20" s="14"/>
-      <c r="D20" s="14"/>
-      <c r="E20" s="14"/>
-      <c r="F20" s="14"/>
-      <c r="G20" s="14"/>
-      <c r="H20" s="14"/>
-      <c r="I20" s="15" t="str">
+      <c r="B20" s="14">
+        <v>480</v>
+      </c>
+      <c r="C20" s="14">
+        <v>90</v>
+      </c>
+      <c r="D20" s="14">
+        <v>60</v>
+      </c>
+      <c r="E20" s="14">
+        <v>90</v>
+      </c>
+      <c r="F20" s="14">
+        <v>250</v>
+      </c>
+      <c r="G20" s="14">
+        <v>5</v>
+      </c>
+      <c r="H20" s="14">
+        <v>120</v>
+      </c>
+      <c r="I20" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J20" s="15" t="str">
+        <v>1090</v>
+      </c>
+      <c r="J20" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K20" s="16"/>
-      <c r="L20" s="16"/>
-      <c r="M20" s="16"/>
-      <c r="N20" s="17"/>
+        <v>350</v>
+      </c>
+      <c r="K20" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="L20" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="M20" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N20" s="17" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A21" s="13"/>
-      <c r="B21" s="14"/>
-      <c r="C21" s="14"/>
-      <c r="D21" s="14"/>
-      <c r="E21" s="14"/>
-      <c r="F21" s="14"/>
-      <c r="G21" s="14"/>
-      <c r="H21" s="14"/>
-      <c r="I21" s="15" t="str">
+      <c r="A21" s="13">
+        <v>46266</v>
+      </c>
+      <c r="B21" s="14">
+        <v>440</v>
+      </c>
+      <c r="C21" s="14">
+        <v>60</v>
+      </c>
+      <c r="D21" s="14">
+        <v>90</v>
+      </c>
+      <c r="E21" s="14">
+        <v>120</v>
+      </c>
+      <c r="F21" s="14">
+        <v>250</v>
+      </c>
+      <c r="G21" s="14">
+        <v>5</v>
+      </c>
+      <c r="H21" s="14">
+        <v>180</v>
+      </c>
+      <c r="I21" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J21" s="15" t="str">
+        <v>1140</v>
+      </c>
+      <c r="J21" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K21" s="16"/>
-      <c r="L21" s="16"/>
-      <c r="M21" s="16"/>
-      <c r="N21" s="17"/>
+        <v>300</v>
+      </c>
+      <c r="K21" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L21" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M21" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N21" s="17" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A22" s="13"/>
-      <c r="B22" s="14"/>
-      <c r="C22" s="14"/>
-      <c r="D22" s="14"/>
-      <c r="E22" s="14"/>
-      <c r="F22" s="14"/>
-      <c r="G22" s="14"/>
-      <c r="H22" s="14"/>
-      <c r="I22" s="15" t="str">
+      <c r="A22" s="13">
+        <v>46267</v>
+      </c>
+      <c r="B22" s="14">
+        <v>470</v>
+      </c>
+      <c r="C22" s="14">
+        <v>60</v>
+      </c>
+      <c r="D22" s="14">
+        <v>45</v>
+      </c>
+      <c r="E22" s="14">
+        <v>100</v>
+      </c>
+      <c r="F22" s="14">
+        <v>300</v>
+      </c>
+      <c r="G22" s="14">
+        <v>6</v>
+      </c>
+      <c r="H22" s="14">
+        <v>180</v>
+      </c>
+      <c r="I22" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J22" s="15" t="str">
+        <v>1155</v>
+      </c>
+      <c r="J22" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K22" s="16"/>
-      <c r="L22" s="16"/>
-      <c r="M22" s="16"/>
-      <c r="N22" s="17"/>
+        <v>285</v>
+      </c>
+      <c r="K22" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="L22" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M22" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N22" s="17" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A23" s="13"/>
-      <c r="B23" s="14"/>
-      <c r="C23" s="14"/>
-      <c r="D23" s="14"/>
-      <c r="E23" s="14"/>
-      <c r="F23" s="14"/>
-      <c r="G23" s="14"/>
-      <c r="H23" s="14"/>
-      <c r="I23" s="15" t="str">
+      <c r="A23" s="13">
+        <v>46268</v>
+      </c>
+      <c r="B23" s="14">
+        <v>430</v>
+      </c>
+      <c r="C23" s="14">
+        <v>60</v>
+      </c>
+      <c r="D23" s="14">
+        <v>60</v>
+      </c>
+      <c r="E23" s="14">
+        <v>80</v>
+      </c>
+      <c r="F23" s="14">
+        <v>300</v>
+      </c>
+      <c r="G23" s="14">
+        <v>6</v>
+      </c>
+      <c r="H23" s="14">
+        <v>120</v>
+      </c>
+      <c r="I23" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J23" s="15" t="str">
+        <v>1050</v>
+      </c>
+      <c r="J23" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K23" s="16"/>
-      <c r="L23" s="16"/>
-      <c r="M23" s="16"/>
-      <c r="N23" s="17"/>
+        <v>390</v>
+      </c>
+      <c r="K23" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="L23" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M23" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N23" s="17" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A24" s="13"/>
-      <c r="B24" s="14"/>
-      <c r="C24" s="14"/>
-      <c r="D24" s="14"/>
-      <c r="E24" s="14"/>
-      <c r="F24" s="14"/>
-      <c r="G24" s="14"/>
-      <c r="H24" s="14"/>
-      <c r="I24" s="15" t="str">
+      <c r="A24" s="13">
+        <v>46269</v>
+      </c>
+      <c r="B24" s="14">
+        <v>420</v>
+      </c>
+      <c r="C24" s="14">
+        <v>80</v>
+      </c>
+      <c r="D24" s="14">
+        <v>70</v>
+      </c>
+      <c r="E24" s="14">
+        <v>120</v>
+      </c>
+      <c r="F24" s="14">
+        <v>300</v>
+      </c>
+      <c r="G24" s="14">
+        <v>6</v>
+      </c>
+      <c r="H24" s="14">
+        <v>150</v>
+      </c>
+      <c r="I24" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J24" s="15" t="str">
+        <v>1140</v>
+      </c>
+      <c r="J24" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K24" s="16"/>
-      <c r="L24" s="16"/>
-      <c r="M24" s="16"/>
-      <c r="N24" s="17"/>
-    </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A25" s="13"/>
-      <c r="B25" s="14"/>
-      <c r="C25" s="14"/>
-      <c r="D25" s="14"/>
-      <c r="E25" s="14"/>
-      <c r="F25" s="14"/>
-      <c r="G25" s="14"/>
-      <c r="H25" s="14"/>
-      <c r="I25" s="15" t="str">
+        <v>300</v>
+      </c>
+      <c r="K24" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="L24" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M24" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N24" s="17" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A25" s="13">
+        <v>46270</v>
+      </c>
+      <c r="B25" s="14">
+        <v>520</v>
+      </c>
+      <c r="C25" s="14">
+        <v>120</v>
+      </c>
+      <c r="D25" s="14">
+        <v>90</v>
+      </c>
+      <c r="E25" s="14">
+        <v>100</v>
+      </c>
+      <c r="F25" s="14">
+        <v>0</v>
+      </c>
+      <c r="G25" s="14">
+        <v>0</v>
+      </c>
+      <c r="H25" s="14">
+        <v>190</v>
+      </c>
+      <c r="I25" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J25" s="15" t="str">
+        <v>1020</v>
+      </c>
+      <c r="J25" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K25" s="16"/>
-      <c r="L25" s="16"/>
-      <c r="M25" s="16"/>
-      <c r="N25" s="17"/>
-    </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A26" s="13"/>
-      <c r="B26" s="14"/>
-      <c r="C26" s="14"/>
-      <c r="D26" s="14"/>
-      <c r="E26" s="14"/>
-      <c r="F26" s="14"/>
-      <c r="G26" s="14"/>
-      <c r="H26" s="14"/>
-      <c r="I26" s="15" t="str">
+        <v>420</v>
+      </c>
+      <c r="K25" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L25" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M25" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N25" s="17" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A26" s="13">
+        <v>46271</v>
+      </c>
+      <c r="B26" s="14">
+        <v>530</v>
+      </c>
+      <c r="C26" s="14">
+        <v>120</v>
+      </c>
+      <c r="D26" s="14">
+        <v>120</v>
+      </c>
+      <c r="E26" s="14">
+        <v>120</v>
+      </c>
+      <c r="F26" s="14">
+        <v>0</v>
+      </c>
+      <c r="G26" s="14">
+        <v>0</v>
+      </c>
+      <c r="H26" s="14">
+        <v>190</v>
+      </c>
+      <c r="I26" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J26" s="15" t="str">
+        <v>1080</v>
+      </c>
+      <c r="J26" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K26" s="16"/>
-      <c r="L26" s="16"/>
-      <c r="M26" s="16"/>
-      <c r="N26" s="17"/>
+        <v>360</v>
+      </c>
+      <c r="K26" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="L26" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M26" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N26" s="17" t="s">
+        <v>83</v>
+      </c>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A27" s="13"/>
-      <c r="B27" s="14"/>
-      <c r="C27" s="14"/>
-      <c r="D27" s="14"/>
-      <c r="E27" s="14"/>
-      <c r="F27" s="14"/>
-      <c r="G27" s="14"/>
-      <c r="H27" s="14"/>
-      <c r="I27" s="15" t="str">
+      <c r="A27" s="13">
+        <v>46272</v>
+      </c>
+      <c r="B27" s="14">
+        <v>430</v>
+      </c>
+      <c r="C27" s="14">
+        <v>90</v>
+      </c>
+      <c r="D27" s="14">
+        <v>60</v>
+      </c>
+      <c r="E27" s="14">
+        <v>80</v>
+      </c>
+      <c r="F27" s="14">
+        <v>250</v>
+      </c>
+      <c r="G27" s="14">
+        <v>5</v>
+      </c>
+      <c r="H27" s="14">
+        <v>180</v>
+      </c>
+      <c r="I27" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J27" s="15" t="str">
+        <v>1090</v>
+      </c>
+      <c r="J27" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K27" s="16"/>
-      <c r="L27" s="16"/>
-      <c r="M27" s="16"/>
-      <c r="N27" s="17"/>
-    </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A28" s="13"/>
-      <c r="B28" s="14"/>
-      <c r="C28" s="14"/>
-      <c r="D28" s="14"/>
-      <c r="E28" s="14"/>
-      <c r="F28" s="14"/>
-      <c r="G28" s="14"/>
-      <c r="H28" s="14"/>
-      <c r="I28" s="15" t="str">
+        <v>350</v>
+      </c>
+      <c r="K27" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L27" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="M27" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N27" s="17" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A28" s="13">
+        <v>46273</v>
+      </c>
+      <c r="B28" s="14">
+        <v>440</v>
+      </c>
+      <c r="C28" s="14">
+        <v>45</v>
+      </c>
+      <c r="D28" s="14">
+        <v>90</v>
+      </c>
+      <c r="E28" s="14">
+        <v>45</v>
+      </c>
+      <c r="F28" s="14">
+        <v>250</v>
+      </c>
+      <c r="G28" s="14">
+        <v>5</v>
+      </c>
+      <c r="H28" s="14">
+        <v>120</v>
+      </c>
+      <c r="I28" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J28" s="15" t="str">
+        <v>990</v>
+      </c>
+      <c r="J28" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K28" s="16"/>
-      <c r="L28" s="16"/>
-      <c r="M28" s="16"/>
-      <c r="N28" s="17"/>
+        <v>450</v>
+      </c>
+      <c r="K28" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="L28" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="M28" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="N28" s="17" t="s">
+        <v>85</v>
+      </c>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A29" s="13"/>
-      <c r="B29" s="14"/>
-      <c r="C29" s="14"/>
-      <c r="D29" s="14"/>
-      <c r="E29" s="14"/>
-      <c r="F29" s="14"/>
-      <c r="G29" s="14"/>
-      <c r="H29" s="14"/>
-      <c r="I29" s="15" t="str">
+      <c r="A29" s="13">
+        <v>46274</v>
+      </c>
+      <c r="B29" s="14">
+        <v>430</v>
+      </c>
+      <c r="C29" s="14">
+        <v>60</v>
+      </c>
+      <c r="D29" s="14">
+        <v>80</v>
+      </c>
+      <c r="E29" s="14">
+        <v>0</v>
+      </c>
+      <c r="F29" s="14">
+        <v>300</v>
+      </c>
+      <c r="G29" s="14">
+        <v>6</v>
+      </c>
+      <c r="H29" s="14">
+        <v>90</v>
+      </c>
+      <c r="I29" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J29" s="15" t="str">
+        <v>960</v>
+      </c>
+      <c r="J29" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K29" s="16"/>
-      <c r="L29" s="16"/>
-      <c r="M29" s="16"/>
-      <c r="N29" s="17"/>
-    </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A30" s="13"/>
-      <c r="B30" s="14"/>
-      <c r="C30" s="14"/>
-      <c r="D30" s="14"/>
-      <c r="E30" s="14"/>
-      <c r="F30" s="14"/>
-      <c r="G30" s="14"/>
-      <c r="H30" s="14"/>
-      <c r="I30" s="15" t="str">
+        <v>480</v>
+      </c>
+      <c r="K29" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L29" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M29" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N29" s="17" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A30" s="13">
+        <v>46275</v>
+      </c>
+      <c r="B30" s="14">
+        <v>450</v>
+      </c>
+      <c r="C30" s="14">
+        <v>80</v>
+      </c>
+      <c r="D30" s="14">
+        <v>40</v>
+      </c>
+      <c r="E30" s="14">
+        <v>30</v>
+      </c>
+      <c r="F30" s="14">
+        <v>300</v>
+      </c>
+      <c r="G30" s="14">
+        <v>6</v>
+      </c>
+      <c r="H30" s="14">
+        <v>120</v>
+      </c>
+      <c r="I30" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J30" s="15" t="str">
+        <v>1020</v>
+      </c>
+      <c r="J30" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K30" s="16"/>
-      <c r="L30" s="16"/>
-      <c r="M30" s="16"/>
-      <c r="N30" s="17"/>
-    </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A31" s="13"/>
-      <c r="B31" s="14"/>
-      <c r="C31" s="14"/>
-      <c r="D31" s="14"/>
-      <c r="E31" s="14"/>
-      <c r="F31" s="14"/>
-      <c r="G31" s="14"/>
-      <c r="H31" s="14"/>
-      <c r="I31" s="15" t="str">
+        <v>420</v>
+      </c>
+      <c r="K30" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="L30" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="M30" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N30" s="17" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A31" s="13">
+        <v>46276</v>
+      </c>
+      <c r="B31" s="14">
+        <v>540</v>
+      </c>
+      <c r="C31" s="14">
+        <v>90</v>
+      </c>
+      <c r="D31" s="14">
+        <v>80</v>
+      </c>
+      <c r="E31" s="14">
+        <v>40</v>
+      </c>
+      <c r="F31" s="14">
+        <v>300</v>
+      </c>
+      <c r="G31" s="14">
+        <v>6</v>
+      </c>
+      <c r="H31" s="14">
+        <v>120</v>
+      </c>
+      <c r="I31" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J31" s="15" t="str">
+        <v>1170</v>
+      </c>
+      <c r="J31" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K31" s="16"/>
-      <c r="L31" s="16"/>
-      <c r="M31" s="16"/>
-      <c r="N31" s="17"/>
+        <v>270</v>
+      </c>
+      <c r="K31" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="L31" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="M31" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="N31" s="17" t="s">
+        <v>88</v>
+      </c>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32" s="13"/>

</xml_diff>